<commit_message>
added cpt code logic
</commit_message>
<xml_diff>
--- a/Macros/dx_code_ref_excel.xlsx
+++ b/Macros/dx_code_ref_excel.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashok\Documents\dheeraj_project\dheeraj_project\Macros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{553A46E3-C0B2-45B7-B657-178E1EA459B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C83F51-AE05-4113-9A49-CF4D6C66A1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="10420" xr2:uid="{2F4E0F0A-CE10-4043-8855-6D7DA4E5309B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="10420" activeTab="1" xr2:uid="{2F4E0F0A-CE10-4043-8855-6D7DA4E5309B}"/>
   </bookViews>
   <sheets>
     <sheet name="dx_code_ref" sheetId="1" r:id="rId1"/>
-    <sheet name="cpt_code_100" sheetId="10" r:id="rId2"/>
-    <sheet name="possible_hcr_list" sheetId="9" r:id="rId3"/>
-    <sheet name="remove_discount_inel" sheetId="8" r:id="rId4"/>
-    <sheet name="apply_discount_after_denial" sheetId="7" r:id="rId5"/>
-    <sheet name="check_inel_code" sheetId="6" r:id="rId6"/>
-    <sheet name="exception_denial_codes" sheetId="5" r:id="rId7"/>
-    <sheet name="cpt_denial" sheetId="4" r:id="rId8"/>
-    <sheet name="rejected" sheetId="3" r:id="rId9"/>
-    <sheet name="cpt_code_price" sheetId="2" r:id="rId10"/>
+    <sheet name="lab_cpt_codes" sheetId="11" r:id="rId2"/>
+    <sheet name="cpt_code_100" sheetId="10" r:id="rId3"/>
+    <sheet name="possible_hcr_list" sheetId="9" r:id="rId4"/>
+    <sheet name="remove_discount_inel" sheetId="8" r:id="rId5"/>
+    <sheet name="apply_discount_after_denial" sheetId="7" r:id="rId6"/>
+    <sheet name="check_inel_code" sheetId="6" r:id="rId7"/>
+    <sheet name="exception_denial_codes" sheetId="5" r:id="rId8"/>
+    <sheet name="cpt_denial" sheetId="4" r:id="rId9"/>
+    <sheet name="rejected" sheetId="3" r:id="rId10"/>
+    <sheet name="cpt_code_price" sheetId="2" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="140">
   <si>
     <t>ICD10-CM DX CODES</t>
   </si>
@@ -439,6 +440,21 @@
   </si>
   <si>
     <t>T5999</t>
+  </si>
+  <si>
+    <t>rule</t>
+  </si>
+  <si>
+    <t>codes</t>
+  </si>
+  <si>
+    <t>rule_991</t>
+  </si>
+  <si>
+    <t>112233
+665544
+998877
+998566</t>
   </si>
 </sst>
 </file>
@@ -922,9 +938,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1285,7 +1304,8 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="25.453125" customWidth="1"/>
+    <col min="1" max="1" width="25.6328125" customWidth="1"/>
+    <col min="2" max="2" width="19.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -1360,6 +1380,61 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A030C989-FE14-4DF9-98F5-0A87EF77C80D}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>947</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{029C2F6A-04DA-490D-B46A-4CF4D7D74C57}">
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1618,6 +1693,36 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92756BA4-5FE7-42B5-8637-B718E53ABDD3}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.36328125" customWidth="1"/>
+    <col min="2" max="2" width="43.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2C3A98-B3F2-4B20-9C61-91803468C444}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1637,7 +1742,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{282E10B9-E08C-4AD4-BD13-D29B0D8F421C}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1692,7 +1797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E14A39E7-4923-4181-A824-E14B7CBFB69C}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1722,7 +1827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{562DC286-2354-4FF3-A45F-D2AF3D30AD28}">
   <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1772,7 +1877,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CFC768-6AB4-40A7-A6EB-C2DA0B6A35D3}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1827,7 +1932,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EAC657B-23D4-4B2C-8DC2-A2AC3FB1DB90}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1862,7 +1967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A86B88A2-811D-489D-ADB3-39882C2D2983}">
   <dimension ref="A1:C271"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3231,59 +3336,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A030C989-FE14-4DF9-98F5-0A87EF77C80D}">
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:1" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>902</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>858</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>947</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>